<commit_message>
Regenerate the ready-made import template with the Round column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFUNdVNXksCb9Katm6q2mb
</commit_message>
<xml_diff>
--- a/zeno-auction/templates/ZenoBid-import-template.xlsx
+++ b/zeno-auction/templates/ZenoBid-import-template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -36,6 +36,9 @@
     <t>Price Paid</t>
   </si>
   <si>
+    <t>Round</t>
+  </si>
+  <si>
     <t>Aarav Mehta</t>
   </si>
   <si>
@@ -69,6 +72,12 @@
     <t>Thunder Hawks</t>
   </si>
   <si>
+    <t>Dev Patel</t>
+  </si>
+  <si>
+    <t>Round 2 example: saved for the next round, hidden until it starts.</t>
+  </si>
+  <si>
     <t>Captain</t>
   </si>
   <si>
@@ -109,6 +118,12 @@
   </si>
   <si>
     <t>7. Re-importing a player with the same Name updates them instead of adding a duplicate.</t>
+  </si>
+  <si>
+    <t>8. Round: leave it empty for players who are up for auction now. Write the NEXT round number (for example 2 while round 1 is on) to save a player for the next round:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   they stay hidden from captains and the big screen, and join the pool when the auctioneer starts that round. Only the very next round can be prepared ahead.</t>
   </si>
   <si>
     <t>In ZenoBid: Players tab → Import Excel → choose this file → check the preview → Import.</t>
@@ -520,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G300"/>
+  <dimension ref="A1:H300"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -532,7 +547,7 @@
     <col min="7" max="7" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -554,67 +569,90 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1">
         <v>2000000</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
         <v>2500000</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1">
         <v>3000000</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G4" s="1">
         <v>12000000</v>
       </c>
     </row>
-    <row r="5" spans="6:6" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2000000</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5">
+        <v>2</v>
+      </c>
+    </row>
     <row r="6" spans="6:6" x14ac:dyDescent="0.25"/>
     <row r="7" spans="6:6" x14ac:dyDescent="0.25"/>
     <row r="8" spans="6:6" x14ac:dyDescent="0.25"/>
@@ -911,7 +949,7 @@
     <row r="299" spans="6:6" x14ac:dyDescent="0.25"/>
     <row r="300" spans="6:6" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Unknown team" error="This team is not on the Teams sheet. Add it there first." sqref="F10:F300">
       <formula1>Teams!$A$2:$A$40</formula1>
@@ -940,18 +978,18 @@
         <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1">
         <v>120000000</v>
@@ -959,10 +997,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1">
         <v>120000000</v>
@@ -976,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -984,67 +1022,77 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>33</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>